<commit_message>
item docs: chorus joins the live-{rank} whitelist (v6.89) — LINT clean
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/item-list.xlsx
+++ b/item-list.xlsx
@@ -7911,7 +7911,7 @@
       </c>
       <c r="P96" s="14" t="inlineStr">
         <is>
-          <t>UNWIRED</t>
+          <t>TEMPLATE</t>
         </is>
       </c>
     </row>
@@ -14329,7 +14329,7 @@
       </c>
       <c r="P31" s="14" t="inlineStr">
         <is>
-          <t>UNWIRED</t>
+          <t>TEMPLATE</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v7.06: Old Joker debt pays in every class (not just pillars); Lone Eye is a plain peek
- rollThirstGifts: drop the tier floor and spread picks across classes. Flat
  rarity (v6.98) left value-3 items as rare-tier only — nearly all pillars — so
  a big debt collapsed to pillars alone (100% pillar-only shelves at budget 12+).
  Now a heavy debt fills a wide, VARIED shelf (a mix of pillar/base/sticker/
  same-power/pack/card), reaching for the dearer item within each fresh class.
- Lone Eye: remove the "only while no Same-Power is equipped" gate — it now just
  peeks the next card. Availability, log line, reason text, description, docs.
- Tests: coat-shelf test now asserts variety (never pillars-only); a new V699
  regression asserts no multi-row debt is pillar-only; Lone Eye validation flips
  to "fires even with a power equipped".

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/item-list.xlsx
+++ b/item-list.xlsx
@@ -553,7 +553,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NINELIVES — item pool (v7.05)</t>
+          <t>NINELIVES — item pool (v7.06)</t>
         </is>
       </c>
     </row>
@@ -7494,7 +7494,7 @@
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t>needs an empty Same-Power slot</t>
+          <t>peek the next card</t>
         </is>
       </c>
       <c r="D91" s="8" t="inlineStr"/>
@@ -7537,7 +7537,7 @@
       <c r="M91" s="8" t="inlineStr"/>
       <c r="N91" s="11" t="inlineStr">
         <is>
-          <t>If no Same-Power is equipped → peek next card</t>
+          <t>Peek the next card</t>
         </is>
       </c>
       <c r="O91" s="9" t="inlineStr">
@@ -14342,7 +14342,7 @@
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t>needs an empty Same-Power slot</t>
+          <t>peek the next card</t>
         </is>
       </c>
       <c r="D81" s="8" t="inlineStr"/>
@@ -14385,7 +14385,7 @@
       <c r="M81" s="8" t="inlineStr"/>
       <c r="N81" s="11" t="inlineStr">
         <is>
-          <t>If no Same-Power is equipped → peek next card</t>
+          <t>Peek the next card</t>
         </is>
       </c>
       <c r="O81" s="9" t="inlineStr">

</xml_diff>